<commit_message>
data: complete English localization for release
- 미번역 영문 77행(스킬 이름·설명·스토리, 신속물약2 설명) 번역
- 영어 대사 71줄에 섞여 있던 한글 아이템·지역명을 영문명으로
- 런타임 하드코딩 한글 → 로컬라이즈 키: 능력 발동 조건(15종, 어순이 달라 서식 키로),
  방치/오프라인 보상 알림, NPC 이름, 고유기술, 미니몬 기본명, 능력 #id, 상점/여정 잠금 사유,
  기본 플레이어 이름 — EnemyEvade/EnemyLowHp 조건이 enum 이름 그대로 찍히던 것도 함께
- 출시 UI 키 추가(설정/게임 종료/크레딧/시스템/전체 화면/뒤로가기 종료 안내/감사 인사/장비 제목)
- 재현: python _tools/fix_english_localization.py [--write|--check] → Tools/ParseAllLocal
  (check: 영문에 한글 0, 영문==한글 0, 중복 키 0, 1945행)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Assets/@Resources/Data/Excel/DialogueData.xlsx
+++ b/Assets/@Resources/Data/Excel/DialogueData.xlsx
@@ -578,7 +578,7 @@
       <c r="C2" t="inlineStr">
         <is>
           <t>Back again.
-Did you bring &lt;color=#2DFF00&gt;&lt;b&gt;5&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;까마귀 깃털&lt;/b&gt;&lt;/color&gt;?</t>
+Did you bring &lt;color=#2DFF00&gt;&lt;b&gt;5&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;Crow Feathers&lt;/b&gt;&lt;/color&gt;?</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
       <c r="C4" t="inlineStr">
         <is>
           <t>A new &lt;color=#00B9FF&gt;Rank 5 Permit&lt;/color&gt; has been issued.
-You may now enter &lt;color=#B0FF06&gt;텅 빈 굴&lt;/color&gt;.
+You may now enter &lt;color=#B0FF06&gt;Hollow Burrow&lt;/color&gt;.
 Recommended level: &lt;color=#FFFF00&gt;49&lt;/color&gt; or higher.</t>
         </is>
       </c>
@@ -635,8 +635,8 @@
       <c r="C5" t="inlineStr">
         <is>
           <t>To reach &lt;color=#00B9FF&gt;rank 6&lt;/color&gt;,
-you will need &lt;color=#2DFF00&gt;&lt;b&gt;7&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;슬라임 젤리&lt;/b&gt;&lt;/color&gt;.
-They drop from the creatures of &lt;color=#B0FF06&gt;텅 빈 굴&lt;/color&gt;.</t>
+you will need &lt;color=#2DFF00&gt;&lt;b&gt;7&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;Slime Jellies&lt;/b&gt;&lt;/color&gt;.
+They drop from the creatures of &lt;color=#B0FF06&gt;Hollow Burrow&lt;/color&gt;.</t>
         </is>
       </c>
     </row>
@@ -699,7 +699,7 @@
       <c r="C2" t="inlineStr">
         <is>
           <t>Back again.
-Did you bring &lt;color=#2DFF00&gt;&lt;b&gt;7&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;슬라임 젤리&lt;/b&gt;&lt;/color&gt;?</t>
+Did you bring &lt;color=#2DFF00&gt;&lt;b&gt;7&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;Slime Jellies&lt;/b&gt;&lt;/color&gt;?</t>
         </is>
       </c>
     </row>
@@ -737,7 +737,7 @@
       <c r="C4" t="inlineStr">
         <is>
           <t>A new &lt;color=#00B9FF&gt;Rank 6 Permit&lt;/color&gt; has been issued.
-You may now enter &lt;color=#B0FF06&gt;소금 늪지&lt;/color&gt;.
+You may now enter &lt;color=#B0FF06&gt;Salt Marsh&lt;/color&gt;.
 Recommended level: &lt;color=#FFFF00&gt;61&lt;/color&gt; or higher.</t>
         </is>
       </c>
@@ -756,8 +756,8 @@
       <c r="C5" t="inlineStr">
         <is>
           <t>To reach &lt;color=#00B9FF&gt;rank 7&lt;/color&gt;,
-you will need &lt;color=#2DFF00&gt;&lt;b&gt;9&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;늑대 송곳니&lt;/b&gt;&lt;/color&gt;.
-They drop from the creatures of &lt;color=#B0FF06&gt;소금 늪지&lt;/color&gt;.</t>
+you will need &lt;color=#2DFF00&gt;&lt;b&gt;9&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;Wolf Fangs&lt;/b&gt;&lt;/color&gt;.
+They drop from the creatures of &lt;color=#B0FF06&gt;Salt Marsh&lt;/color&gt;.</t>
         </is>
       </c>
     </row>
@@ -820,7 +820,7 @@
       <c r="C2" t="inlineStr">
         <is>
           <t>Back again.
-Did you bring &lt;color=#2DFF00&gt;&lt;b&gt;9&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;늑대 송곳니&lt;/b&gt;&lt;/color&gt;?</t>
+Did you bring &lt;color=#2DFF00&gt;&lt;b&gt;9&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;Wolf Fangs&lt;/b&gt;&lt;/color&gt;?</t>
         </is>
       </c>
     </row>
@@ -858,7 +858,7 @@
       <c r="C4" t="inlineStr">
         <is>
           <t>A new &lt;color=#00B9FF&gt;Rank 7 Permit&lt;/color&gt; has been issued.
-You may now enter &lt;color=#B0FF06&gt;밀물 동굴&lt;/color&gt;.
+You may now enter &lt;color=#B0FF06&gt;Tidal Cavern&lt;/color&gt;.
 Recommended level: &lt;color=#FFFF00&gt;73&lt;/color&gt; or higher.</t>
         </is>
       </c>
@@ -877,8 +877,8 @@
       <c r="C5" t="inlineStr">
         <is>
           <t>To reach &lt;color=#00B9FF&gt;rank 8&lt;/color&gt;,
-you will need &lt;color=#2DFF00&gt;&lt;b&gt;9&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;멧돼지 가죽&lt;/b&gt;&lt;/color&gt;.
-They drop from the creatures of &lt;color=#B0FF06&gt;밀물 동굴&lt;/color&gt;.</t>
+you will need &lt;color=#2DFF00&gt;&lt;b&gt;9&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;Boar Hides&lt;/b&gt;&lt;/color&gt;.
+They drop from the creatures of &lt;color=#B0FF06&gt;Tidal Cavern&lt;/color&gt;.</t>
         </is>
       </c>
     </row>
@@ -941,7 +941,7 @@
       <c r="C2" t="inlineStr">
         <is>
           <t>Back again.
-Did you bring &lt;color=#2DFF00&gt;&lt;b&gt;9&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;멧돼지 가죽&lt;/b&gt;&lt;/color&gt;?</t>
+Did you bring &lt;color=#2DFF00&gt;&lt;b&gt;9&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;Boar Hides&lt;/b&gt;&lt;/color&gt;?</t>
         </is>
       </c>
     </row>
@@ -979,7 +979,7 @@
       <c r="C4" t="inlineStr">
         <is>
           <t>A new &lt;color=#00B9FF&gt;Rank 8 Permit&lt;/color&gt; has been issued.
-You may now enter &lt;color=#B0FF06&gt;부서진 잔교&lt;/color&gt;.
+You may now enter &lt;color=#B0FF06&gt;Broken Pier&lt;/color&gt;.
 Recommended level: &lt;color=#FFFF00&gt;85&lt;/color&gt; or higher.</t>
         </is>
       </c>
@@ -998,8 +998,8 @@
       <c r="C5" t="inlineStr">
         <is>
           <t>To reach &lt;color=#00B9FF&gt;rank 9&lt;/color&gt;,
-you will need &lt;color=#2DFF00&gt;&lt;b&gt;11&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;거미 실크&lt;/b&gt;&lt;/color&gt;.
-They drop from the creatures of &lt;color=#B0FF06&gt;부서진 잔교&lt;/color&gt;.</t>
+you will need &lt;color=#2DFF00&gt;&lt;b&gt;11&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;Spider Silk&lt;/b&gt;&lt;/color&gt;.
+They drop from the creatures of &lt;color=#B0FF06&gt;Broken Pier&lt;/color&gt;.</t>
         </is>
       </c>
     </row>
@@ -1062,7 +1062,7 @@
       <c r="C2" t="inlineStr">
         <is>
           <t>Back again.
-Did you bring &lt;color=#2DFF00&gt;&lt;b&gt;11&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;거미 실크&lt;/b&gt;&lt;/color&gt;?</t>
+Did you bring &lt;color=#2DFF00&gt;&lt;b&gt;11&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;Spider Silk&lt;/b&gt;&lt;/color&gt;?</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1100,7 @@
       <c r="C4" t="inlineStr">
         <is>
           <t>A new &lt;color=#00B9FF&gt;Rank 9 Permit&lt;/color&gt; has been issued.
-You may now enter &lt;color=#B0FF06&gt;폭풍 절벽&lt;/color&gt;.
+You may now enter &lt;color=#B0FF06&gt;Storm Cliff&lt;/color&gt;.
 Recommended level: &lt;color=#FFFF00&gt;97&lt;/color&gt; or higher.</t>
         </is>
       </c>
@@ -1119,8 +1119,8 @@
       <c r="C5" t="inlineStr">
         <is>
           <t>To reach &lt;color=#00B9FF&gt;rank 10&lt;/color&gt;,
-you will need &lt;color=#2DFF00&gt;&lt;b&gt;11&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;바람 정수&lt;/b&gt;&lt;/color&gt;.
-They drop from the creatures of &lt;color=#B0FF06&gt;폭풍 절벽&lt;/color&gt;.</t>
+you will need &lt;color=#2DFF00&gt;&lt;b&gt;11&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;Wind Essence&lt;/b&gt;&lt;/color&gt;.
+They drop from the creatures of &lt;color=#B0FF06&gt;Storm Cliff&lt;/color&gt;.</t>
         </is>
       </c>
     </row>
@@ -1183,7 +1183,7 @@
       <c r="C2" t="inlineStr">
         <is>
           <t>Back again.
-Did you bring &lt;color=#2DFF00&gt;&lt;b&gt;11&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;바람 정수&lt;/b&gt;&lt;/color&gt;?</t>
+Did you bring &lt;color=#2DFF00&gt;&lt;b&gt;11&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;Wind Essence&lt;/b&gt;&lt;/color&gt;?</t>
         </is>
       </c>
     </row>
@@ -1221,7 +1221,7 @@
       <c r="C4" t="inlineStr">
         <is>
           <t>A new &lt;color=#00B9FF&gt;Rank 10 Permit&lt;/color&gt; has been issued.
-You may now enter &lt;color=#B0FF06&gt;표류목 숲&lt;/color&gt;.
+You may now enter &lt;color=#B0FF06&gt;Driftwood Wood&lt;/color&gt;.
 Recommended level: &lt;color=#FFFF00&gt;109&lt;/color&gt; or higher.</t>
         </is>
       </c>
@@ -1240,8 +1240,8 @@
       <c r="C5" t="inlineStr">
         <is>
           <t>To reach &lt;color=#00B9FF&gt;rank 11&lt;/color&gt;,
-you will need &lt;color=#2DFF00&gt;&lt;b&gt;13&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;그림자 응결물&lt;/b&gt;&lt;/color&gt;.
-They drop from the creatures of &lt;color=#B0FF06&gt;표류목 숲&lt;/color&gt;.</t>
+you will need &lt;color=#2DFF00&gt;&lt;b&gt;13&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;Shadow Clots&lt;/b&gt;&lt;/color&gt;.
+They drop from the creatures of &lt;color=#B0FF06&gt;Driftwood Wood&lt;/color&gt;.</t>
         </is>
       </c>
     </row>
@@ -1304,7 +1304,7 @@
       <c r="C2" t="inlineStr">
         <is>
           <t>Back again.
-Did you bring &lt;color=#2DFF00&gt;&lt;b&gt;13&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;그림자 응결물&lt;/b&gt;&lt;/color&gt;?</t>
+Did you bring &lt;color=#2DFF00&gt;&lt;b&gt;13&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;Shadow Clots&lt;/b&gt;&lt;/color&gt;?</t>
         </is>
       </c>
     </row>
@@ -1342,7 +1342,7 @@
       <c r="C4" t="inlineStr">
         <is>
           <t>A new &lt;color=#00B9FF&gt;Rank 11 Permit&lt;/color&gt; has been issued.
-You may now enter &lt;color=#B0FF06&gt;잿불 구덩이&lt;/color&gt;.
+You may now enter &lt;color=#B0FF06&gt;Cinder Pit&lt;/color&gt;.
 Recommended level: &lt;color=#FFFF00&gt;121&lt;/color&gt; or higher.</t>
         </is>
       </c>
@@ -1361,8 +1361,8 @@
       <c r="C5" t="inlineStr">
         <is>
           <t>To reach &lt;color=#00B9FF&gt;rank 12&lt;/color&gt;,
-you will need &lt;color=#2DFF00&gt;&lt;b&gt;15&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;박쥐 날개막&lt;/b&gt;&lt;/color&gt;.
-They drop from the creatures of &lt;color=#B0FF06&gt;잿불 구덩이&lt;/color&gt;.</t>
+you will need &lt;color=#2DFF00&gt;&lt;b&gt;15&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;Bat Membranes&lt;/b&gt;&lt;/color&gt;.
+They drop from the creatures of &lt;color=#B0FF06&gt;Cinder Pit&lt;/color&gt;.</t>
         </is>
       </c>
     </row>
@@ -1425,7 +1425,7 @@
       <c r="C2" t="inlineStr">
         <is>
           <t>Back again.
-Did you bring &lt;color=#2DFF00&gt;&lt;b&gt;15&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;박쥐 날개막&lt;/b&gt;&lt;/color&gt;?</t>
+Did you bring &lt;color=#2DFF00&gt;&lt;b&gt;15&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;Bat Membranes&lt;/b&gt;&lt;/color&gt;?</t>
         </is>
       </c>
     </row>
@@ -1463,7 +1463,7 @@
       <c r="C4" t="inlineStr">
         <is>
           <t>A new &lt;color=#00B9FF&gt;Rank 12 Permit&lt;/color&gt; has been issued.
-You may now enter &lt;color=#B0FF06&gt;깊은 수직굴&lt;/color&gt;.
+You may now enter &lt;color=#B0FF06&gt;Deep Shaft&lt;/color&gt;.
 Recommended level: &lt;color=#FFFF00&gt;133&lt;/color&gt; or higher.</t>
         </is>
       </c>
@@ -1482,8 +1482,8 @@
       <c r="C5" t="inlineStr">
         <is>
           <t>To reach &lt;color=#00B9FF&gt;rank 13&lt;/color&gt;,
-you will need &lt;color=#2DFF00&gt;&lt;b&gt;15&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;수정 파편&lt;/b&gt;&lt;/color&gt;.
-They drop from the creatures of &lt;color=#B0FF06&gt;깊은 수직굴&lt;/color&gt;.</t>
+you will need &lt;color=#2DFF00&gt;&lt;b&gt;15&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;Crystal Shards&lt;/b&gt;&lt;/color&gt;.
+They drop from the creatures of &lt;color=#B0FF06&gt;Deep Shaft&lt;/color&gt;.</t>
         </is>
       </c>
     </row>
@@ -1546,7 +1546,7 @@
       <c r="C2" t="inlineStr">
         <is>
           <t>Back again.
-Did you bring &lt;color=#2DFF00&gt;&lt;b&gt;15&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;수정 파편&lt;/b&gt;&lt;/color&gt;?</t>
+Did you bring &lt;color=#2DFF00&gt;&lt;b&gt;15&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;Crystal Shards&lt;/b&gt;&lt;/color&gt;?</t>
         </is>
       </c>
     </row>
@@ -1584,7 +1584,7 @@
       <c r="C4" t="inlineStr">
         <is>
           <t>A new &lt;color=#00B9FF&gt;Rank 13 Permit&lt;/color&gt; has been issued.
-You may now enter &lt;color=#B0FF06&gt;녹슨 회랑&lt;/color&gt;.
+You may now enter &lt;color=#B0FF06&gt;Rust Hall&lt;/color&gt;.
 Recommended level: &lt;color=#FFFF00&gt;145&lt;/color&gt; or higher.</t>
         </is>
       </c>
@@ -1603,8 +1603,8 @@
       <c r="C5" t="inlineStr">
         <is>
           <t>To reach &lt;color=#00B9FF&gt;rank 14&lt;/color&gt;,
-you will need &lt;color=#2DFF00&gt;&lt;b&gt;17&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;석상 조각&lt;/b&gt;&lt;/color&gt;.
-They drop from the creatures of &lt;color=#B0FF06&gt;녹슨 회랑&lt;/color&gt;.</t>
+you will need &lt;color=#2DFF00&gt;&lt;b&gt;17&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;Statue Fragments&lt;/b&gt;&lt;/color&gt;.
+They drop from the creatures of &lt;color=#B0FF06&gt;Rust Hall&lt;/color&gt;.</t>
         </is>
       </c>
     </row>
@@ -1667,7 +1667,7 @@
       <c r="C2" t="inlineStr">
         <is>
           <t>Back again.
-Did you bring &lt;color=#2DFF00&gt;&lt;b&gt;17&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;석상 조각&lt;/b&gt;&lt;/color&gt;?</t>
+Did you bring &lt;color=#2DFF00&gt;&lt;b&gt;17&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;Statue Fragments&lt;/b&gt;&lt;/color&gt;?</t>
         </is>
       </c>
     </row>
@@ -1705,7 +1705,7 @@
       <c r="C4" t="inlineStr">
         <is>
           <t>A new &lt;color=#00B9FF&gt;Rank 14 Permit&lt;/color&gt; has been issued.
-You may now enter &lt;color=#B0FF06&gt;불씨 광맥&lt;/color&gt;.
+You may now enter &lt;color=#B0FF06&gt;Ember Vein&lt;/color&gt;.
 Recommended level: &lt;color=#FFFF00&gt;157&lt;/color&gt; or higher.</t>
         </is>
       </c>
@@ -1724,8 +1724,8 @@
       <c r="C5" t="inlineStr">
         <is>
           <t>To reach &lt;color=#00B9FF&gt;rank 15&lt;/color&gt;,
-you will need &lt;color=#2DFF00&gt;&lt;b&gt;17&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;광부의 유품&lt;/b&gt;&lt;/color&gt;.
-They drop from the creatures of &lt;color=#B0FF06&gt;불씨 광맥&lt;/color&gt;.</t>
+you will need &lt;color=#2DFF00&gt;&lt;b&gt;17&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;Miner's Relics&lt;/b&gt;&lt;/color&gt;.
+They drop from the creatures of &lt;color=#B0FF06&gt;Ember Vein&lt;/color&gt;.</t>
         </is>
       </c>
     </row>
@@ -1985,7 +1985,7 @@
       <c r="C2" t="inlineStr">
         <is>
           <t>Back again.
-Did you bring &lt;color=#2DFF00&gt;&lt;b&gt;17&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;광부의 유품&lt;/b&gt;&lt;/color&gt;?</t>
+Did you bring &lt;color=#2DFF00&gt;&lt;b&gt;17&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;Miner's Relics&lt;/b&gt;&lt;/color&gt;?</t>
         </is>
       </c>
     </row>
@@ -2023,7 +2023,7 @@
       <c r="C4" t="inlineStr">
         <is>
           <t>A new &lt;color=#00B9FF&gt;Rank 15 Permit&lt;/color&gt; has been issued.
-You may now enter &lt;color=#B0FF06&gt;무너진 갱도&lt;/color&gt;.
+You may now enter &lt;color=#B0FF06&gt;Collapsed Tunnel&lt;/color&gt;.
 Recommended level: &lt;color=#FFFF00&gt;169&lt;/color&gt; or higher.</t>
         </is>
       </c>
@@ -2042,8 +2042,8 @@
       <c r="C5" t="inlineStr">
         <is>
           <t>To reach &lt;color=#00B9FF&gt;rank 16&lt;/color&gt;,
-you will need &lt;color=#2DFF00&gt;&lt;b&gt;19&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;젖은 이끼&lt;/b&gt;&lt;/color&gt;.
-They drop from the creatures of &lt;color=#B0FF06&gt;무너진 갱도&lt;/color&gt;.</t>
+you will need &lt;color=#2DFF00&gt;&lt;b&gt;19&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;Damp Moss&lt;/b&gt;&lt;/color&gt;.
+They drop from the creatures of &lt;color=#B0FF06&gt;Collapsed Tunnel&lt;/color&gt;.</t>
         </is>
       </c>
     </row>
@@ -2106,7 +2106,7 @@
       <c r="C2" t="inlineStr">
         <is>
           <t>Back again.
-Did you bring &lt;color=#2DFF00&gt;&lt;b&gt;19&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;젖은 이끼&lt;/b&gt;&lt;/color&gt;?</t>
+Did you bring &lt;color=#2DFF00&gt;&lt;b&gt;19&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;Damp Moss&lt;/b&gt;&lt;/color&gt;?</t>
         </is>
       </c>
     </row>
@@ -2144,7 +2144,7 @@
       <c r="C4" t="inlineStr">
         <is>
           <t>A new &lt;color=#00B9FF&gt;Rank 16 Permit&lt;/color&gt; has been issued.
-You may now enter &lt;color=#B0FF06&gt;서리 수림&lt;/color&gt;.
+You may now enter &lt;color=#B0FF06&gt;Frost Wood&lt;/color&gt;.
 Recommended level: &lt;color=#FFFF00&gt;181&lt;/color&gt; or higher.</t>
         </is>
       </c>
@@ -2163,8 +2163,8 @@
       <c r="C5" t="inlineStr">
         <is>
           <t>To reach &lt;color=#00B9FF&gt;rank 17&lt;/color&gt;,
-you will need &lt;color=#2DFF00&gt;&lt;b&gt;21&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;박쥐 날개막&lt;/b&gt;&lt;/color&gt;.
-They drop from the creatures of &lt;color=#B0FF06&gt;서리 수림&lt;/color&gt;.</t>
+you will need &lt;color=#2DFF00&gt;&lt;b&gt;21&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;Bat Membranes&lt;/b&gt;&lt;/color&gt;.
+They drop from the creatures of &lt;color=#B0FF06&gt;Frost Wood&lt;/color&gt;.</t>
         </is>
       </c>
     </row>
@@ -2227,7 +2227,7 @@
       <c r="C2" t="inlineStr">
         <is>
           <t>Back again.
-Did you bring &lt;color=#2DFF00&gt;&lt;b&gt;21&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;박쥐 날개막&lt;/b&gt;&lt;/color&gt;?</t>
+Did you bring &lt;color=#2DFF00&gt;&lt;b&gt;21&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;Bat Membranes&lt;/b&gt;&lt;/color&gt;?</t>
         </is>
       </c>
     </row>
@@ -2265,7 +2265,7 @@
       <c r="C4" t="inlineStr">
         <is>
           <t>A new &lt;color=#00B9FF&gt;Rank 17 Permit&lt;/color&gt; has been issued.
-You may now enter &lt;color=#B0FF06&gt;빙하 동굴&lt;/color&gt;.
+You may now enter &lt;color=#B0FF06&gt;Glacier Cave&lt;/color&gt;.
 Recommended level: &lt;color=#FFFF00&gt;193&lt;/color&gt; or higher.</t>
         </is>
       </c>
@@ -2284,8 +2284,8 @@
       <c r="C5" t="inlineStr">
         <is>
           <t>To reach &lt;color=#00B9FF&gt;rank 18&lt;/color&gt;,
-you will need &lt;color=#2DFF00&gt;&lt;b&gt;21&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;두더지 발톱&lt;/b&gt;&lt;/color&gt;.
-They drop from the creatures of &lt;color=#B0FF06&gt;빙하 동굴&lt;/color&gt;.</t>
+you will need &lt;color=#2DFF00&gt;&lt;b&gt;21&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;Mole Claws&lt;/b&gt;&lt;/color&gt;.
+They drop from the creatures of &lt;color=#B0FF06&gt;Glacier Cave&lt;/color&gt;.</t>
         </is>
       </c>
     </row>
@@ -2348,7 +2348,7 @@
       <c r="C2" t="inlineStr">
         <is>
           <t>Back again.
-Did you bring &lt;color=#2DFF00&gt;&lt;b&gt;21&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;두더지 발톱&lt;/b&gt;&lt;/color&gt;?</t>
+Did you bring &lt;color=#2DFF00&gt;&lt;b&gt;21&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;Mole Claws&lt;/b&gt;&lt;/color&gt;?</t>
         </is>
       </c>
     </row>
@@ -2386,7 +2386,7 @@
       <c r="C4" t="inlineStr">
         <is>
           <t>A new &lt;color=#00B9FF&gt;Rank 18 Permit&lt;/color&gt; has been issued.
-You may now enter &lt;color=#B0FF06&gt;고요한 예배당&lt;/color&gt;.
+You may now enter &lt;color=#B0FF06&gt;Silent Chapel&lt;/color&gt;.
 Recommended level: &lt;color=#FFFF00&gt;205&lt;/color&gt; or higher.</t>
         </is>
       </c>
@@ -2405,8 +2405,8 @@
       <c r="C5" t="inlineStr">
         <is>
           <t>To reach &lt;color=#00B9FF&gt;rank 19&lt;/color&gt;,
-you will need &lt;color=#2DFF00&gt;&lt;b&gt;23&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;망령의 재&lt;/b&gt;&lt;/color&gt;.
-They drop from the creatures of &lt;color=#B0FF06&gt;고요한 예배당&lt;/color&gt;.</t>
+you will need &lt;color=#2DFF00&gt;&lt;b&gt;23&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;Revenant Ash&lt;/b&gt;&lt;/color&gt;.
+They drop from the creatures of &lt;color=#B0FF06&gt;Silent Chapel&lt;/color&gt;.</t>
         </is>
       </c>
     </row>
@@ -2469,7 +2469,7 @@
       <c r="C2" t="inlineStr">
         <is>
           <t>Back again.
-Did you bring &lt;color=#2DFF00&gt;&lt;b&gt;23&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;망령의 재&lt;/b&gt;&lt;/color&gt;?</t>
+Did you bring &lt;color=#2DFF00&gt;&lt;b&gt;23&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;Revenant Ash&lt;/b&gt;&lt;/color&gt;?</t>
         </is>
       </c>
     </row>
@@ -2507,7 +2507,7 @@
       <c r="C4" t="inlineStr">
         <is>
           <t>A new &lt;color=#00B9FF&gt;Rank 19 Permit&lt;/color&gt; has been issued.
-You may now enter &lt;color=#B0FF06&gt;새하얀 황야&lt;/color&gt;.
+You may now enter &lt;color=#B0FF06&gt;White Waste&lt;/color&gt;.
 Recommended level: &lt;color=#FFFF00&gt;217&lt;/color&gt; or higher.</t>
         </is>
       </c>
@@ -2526,8 +2526,8 @@
       <c r="C5" t="inlineStr">
         <is>
           <t>To reach &lt;color=#00B9FF&gt;rank 20&lt;/color&gt;,
-you will need &lt;color=#2DFF00&gt;&lt;b&gt;23&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;기사의 문장&lt;/b&gt;&lt;/color&gt;.
-They drop from the creatures of &lt;color=#B0FF06&gt;새하얀 황야&lt;/color&gt;.</t>
+you will need &lt;color=#2DFF00&gt;&lt;b&gt;23&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;Knight's Crests&lt;/b&gt;&lt;/color&gt;.
+They drop from the creatures of &lt;color=#B0FF06&gt;White Waste&lt;/color&gt;.</t>
         </is>
       </c>
     </row>
@@ -2590,7 +2590,7 @@
       <c r="C2" t="inlineStr">
         <is>
           <t>Back again.
-Did you bring &lt;color=#2DFF00&gt;&lt;b&gt;23&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;기사의 문장&lt;/b&gt;&lt;/color&gt;?</t>
+Did you bring &lt;color=#2DFF00&gt;&lt;b&gt;23&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;Knight's Crests&lt;/b&gt;&lt;/color&gt;?</t>
         </is>
       </c>
     </row>
@@ -2628,7 +2628,7 @@
       <c r="C4" t="inlineStr">
         <is>
           <t>A new &lt;color=#00B9FF&gt;Rank 20 Permit&lt;/color&gt; has been issued.
-You may now enter &lt;color=#B0FF06&gt;얼어붙은 금고&lt;/color&gt;.
+You may now enter &lt;color=#B0FF06&gt;Frozen Vault&lt;/color&gt;.
 Recommended level: &lt;color=#FFFF00&gt;229&lt;/color&gt; or higher.</t>
         </is>
       </c>
@@ -2647,8 +2647,8 @@
       <c r="C5" t="inlineStr">
         <is>
           <t>To reach &lt;color=#00B9FF&gt;rank 21&lt;/color&gt;,
-you will need &lt;color=#2DFF00&gt;&lt;b&gt;25&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;수호자의 핵&lt;/b&gt;&lt;/color&gt;.
-They drop from the creatures of &lt;color=#B0FF06&gt;얼어붙은 금고&lt;/color&gt;.</t>
+you will need &lt;color=#2DFF00&gt;&lt;b&gt;25&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;Warden Cores&lt;/b&gt;&lt;/color&gt;.
+They drop from the creatures of &lt;color=#B0FF06&gt;Frozen Vault&lt;/color&gt;.</t>
         </is>
       </c>
     </row>
@@ -2711,7 +2711,7 @@
       <c r="C2" t="inlineStr">
         <is>
           <t>Back again.
-Did you bring &lt;color=#2DFF00&gt;&lt;b&gt;25&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;수호자의 핵&lt;/b&gt;&lt;/color&gt;?</t>
+Did you bring &lt;color=#2DFF00&gt;&lt;b&gt;25&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;Warden Cores&lt;/b&gt;&lt;/color&gt;?</t>
         </is>
       </c>
     </row>
@@ -2749,7 +2749,7 @@
       <c r="C4" t="inlineStr">
         <is>
           <t>A new &lt;color=#00B9FF&gt;Rank 21 Permit&lt;/color&gt; has been issued.
-You may now enter &lt;color=#B0FF06&gt;여명의 정원&lt;/color&gt;.
+You may now enter &lt;color=#B0FF06&gt;Dawn Garden&lt;/color&gt;.
 Recommended level: &lt;color=#FFFF00&gt;241&lt;/color&gt; or higher.</t>
         </is>
       </c>
@@ -2768,8 +2768,8 @@
       <c r="C5" t="inlineStr">
         <is>
           <t>To reach &lt;color=#00B9FF&gt;rank 22&lt;/color&gt;,
-you will need &lt;color=#2DFF00&gt;&lt;b&gt;27&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;망령의 재&lt;/b&gt;&lt;/color&gt;.
-They drop from the creatures of &lt;color=#B0FF06&gt;여명의 정원&lt;/color&gt;.</t>
+you will need &lt;color=#2DFF00&gt;&lt;b&gt;27&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;Revenant Ash&lt;/b&gt;&lt;/color&gt;.
+They drop from the creatures of &lt;color=#B0FF06&gt;Dawn Garden&lt;/color&gt;.</t>
         </is>
       </c>
     </row>
@@ -2832,7 +2832,7 @@
       <c r="C2" t="inlineStr">
         <is>
           <t>Back again.
-Did you bring &lt;color=#2DFF00&gt;&lt;b&gt;27&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;망령의 재&lt;/b&gt;&lt;/color&gt;?</t>
+Did you bring &lt;color=#2DFF00&gt;&lt;b&gt;27&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;Revenant Ash&lt;/b&gt;&lt;/color&gt;?</t>
         </is>
       </c>
     </row>
@@ -2870,7 +2870,7 @@
       <c r="C4" t="inlineStr">
         <is>
           <t>A new &lt;color=#00B9FF&gt;Rank 22 Permit&lt;/color&gt; has been issued.
-You may now enter &lt;color=#B0FF06&gt;공허의 계단&lt;/color&gt;.
+You may now enter &lt;color=#B0FF06&gt;Void Stair&lt;/color&gt;.
 Recommended level: &lt;color=#FFFF00&gt;253&lt;/color&gt; or higher.</t>
         </is>
       </c>
@@ -2889,8 +2889,8 @@
       <c r="C5" t="inlineStr">
         <is>
           <t>To reach &lt;color=#00B9FF&gt;rank 23&lt;/color&gt;,
-you will need &lt;color=#2DFF00&gt;&lt;b&gt;27&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;키메라 갈기&lt;/b&gt;&lt;/color&gt;.
-They drop from the creatures of &lt;color=#B0FF06&gt;공허의 계단&lt;/color&gt;.</t>
+you will need &lt;color=#2DFF00&gt;&lt;b&gt;27&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;Chimera Manes&lt;/b&gt;&lt;/color&gt;.
+They drop from the creatures of &lt;color=#B0FF06&gt;Void Stair&lt;/color&gt;.</t>
         </is>
       </c>
     </row>
@@ -2953,7 +2953,7 @@
       <c r="C2" t="inlineStr">
         <is>
           <t>Back again.
-Did you bring &lt;color=#2DFF00&gt;&lt;b&gt;27&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;키메라 갈기&lt;/b&gt;&lt;/color&gt;?</t>
+Did you bring &lt;color=#2DFF00&gt;&lt;b&gt;27&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;Chimera Manes&lt;/b&gt;&lt;/color&gt;?</t>
         </is>
       </c>
     </row>
@@ -2991,7 +2991,7 @@
       <c r="C4" t="inlineStr">
         <is>
           <t>A new &lt;color=#00B9FF&gt;Rank 23 Permit&lt;/color&gt; has been issued.
-You may now enter &lt;color=#B0FF06&gt;별의 성소&lt;/color&gt;.
+You may now enter &lt;color=#B0FF06&gt;Star Sanctum&lt;/color&gt;.
 Recommended level: &lt;color=#FFFF00&gt;265&lt;/color&gt; or higher.</t>
         </is>
       </c>
@@ -3010,8 +3010,8 @@
       <c r="C5" t="inlineStr">
         <is>
           <t>To reach &lt;color=#00B9FF&gt;rank 24&lt;/color&gt;,
-you will need &lt;color=#2DFF00&gt;&lt;b&gt;29&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;기사의 문장&lt;/b&gt;&lt;/color&gt;.
-They drop from the creatures of &lt;color=#B0FF06&gt;별의 성소&lt;/color&gt;.</t>
+you will need &lt;color=#2DFF00&gt;&lt;b&gt;29&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;Knight's Crests&lt;/b&gt;&lt;/color&gt;.
+They drop from the creatures of &lt;color=#B0FF06&gt;Star Sanctum&lt;/color&gt;.</t>
         </is>
       </c>
     </row>
@@ -3074,7 +3074,7 @@
       <c r="C2" t="inlineStr">
         <is>
           <t>Back again.
-Did you bring &lt;color=#2DFF00&gt;&lt;b&gt;29&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;기사의 문장&lt;/b&gt;&lt;/color&gt;?</t>
+Did you bring &lt;color=#2DFF00&gt;&lt;b&gt;29&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;Knight's Crests&lt;/b&gt;&lt;/color&gt;?</t>
         </is>
       </c>
     </row>
@@ -3112,7 +3112,7 @@
       <c r="C4" t="inlineStr">
         <is>
           <t>A new &lt;color=#00B9FF&gt;Rank 24 Permit&lt;/color&gt; has been issued.
-You may now enter &lt;color=#B0FF06&gt;마지막 성벽&lt;/color&gt;.
+You may now enter &lt;color=#B0FF06&gt;Last Rampart&lt;/color&gt;.
 Recommended level: &lt;color=#FFFF00&gt;277&lt;/color&gt; or higher.</t>
         </is>
       </c>
@@ -3131,8 +3131,8 @@
       <c r="C5" t="inlineStr">
         <is>
           <t>To reach &lt;color=#00B9FF&gt;rank 25&lt;/color&gt;,
-you will need &lt;color=#2DFF00&gt;&lt;b&gt;29&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;수호자의 핵&lt;/b&gt;&lt;/color&gt;.
-They drop from the creatures of &lt;color=#B0FF06&gt;마지막 성벽&lt;/color&gt;.</t>
+you will need &lt;color=#2DFF00&gt;&lt;b&gt;29&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;Warden Cores&lt;/b&gt;&lt;/color&gt;.
+They drop from the creatures of &lt;color=#B0FF06&gt;Last Rampart&lt;/color&gt;.</t>
         </is>
       </c>
     </row>
@@ -3288,7 +3288,7 @@
       <c r="C2" t="inlineStr">
         <is>
           <t>Back again.
-Did you bring &lt;color=#2DFF00&gt;&lt;b&gt;29&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;수호자의 핵&lt;/b&gt;&lt;/color&gt;?</t>
+Did you bring &lt;color=#2DFF00&gt;&lt;b&gt;29&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;Warden Cores&lt;/b&gt;&lt;/color&gt;?</t>
         </is>
       </c>
     </row>
@@ -3326,7 +3326,7 @@
       <c r="C4" t="inlineStr">
         <is>
           <t>A new &lt;color=#00B9FF&gt;Rank 25 Permit&lt;/color&gt; has been issued.
-You may now enter &lt;color=#B0FF06&gt;여명의 왕좌&lt;/color&gt;.
+You may now enter &lt;color=#B0FF06&gt;Throne of Dawn&lt;/color&gt;.
 Recommended level: &lt;color=#FFFF00&gt;289&lt;/color&gt; or higher.</t>
         </is>
       </c>
@@ -3345,8 +3345,8 @@
       <c r="C5" t="inlineStr">
         <is>
           <t>To reach &lt;color=#00B9FF&gt;rank 26&lt;/color&gt;,
-you will need &lt;color=#2DFF00&gt;&lt;b&gt;31&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;망령의 재&lt;/b&gt;&lt;/color&gt;.
-They drop from the creatures of &lt;color=#B0FF06&gt;여명의 왕좌&lt;/color&gt;.</t>
+you will need &lt;color=#2DFF00&gt;&lt;b&gt;31&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;Revenant Ash&lt;/b&gt;&lt;/color&gt;.
+They drop from the creatures of &lt;color=#B0FF06&gt;Throne of Dawn&lt;/color&gt;.</t>
         </is>
       </c>
     </row>
@@ -3409,7 +3409,7 @@
       <c r="C2" t="inlineStr">
         <is>
           <t>Back again.
-Did you bring &lt;color=#2DFF00&gt;&lt;b&gt;31&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;망령의 재&lt;/b&gt;&lt;/color&gt;?</t>
+Did you bring &lt;color=#2DFF00&gt;&lt;b&gt;31&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;Revenant Ash&lt;/b&gt;&lt;/color&gt;?</t>
         </is>
       </c>
     </row>
@@ -4294,8 +4294,8 @@
       <c r="C5" t="inlineStr">
         <is>
           <t>Congratulations on your promotion to a &lt;color=#00B9FF&gt;[&lt;color=#858585&gt;2&lt;/color&gt;]-rank Adventurer&lt;/color&gt;.
-Access to &lt;color=#B0FF06&gt;속삭이는 동굴&lt;/color&gt; has been granted.
-To reach &lt;color=#00B9FF&gt;rank 3&lt;/color&gt;, you will need &lt;color=#2DFF00&gt;&lt;b&gt;3&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;슬라임 젤리&lt;/b&gt;&lt;/color&gt;.</t>
+Access to &lt;color=#B0FF06&gt;Whispering Cave&lt;/color&gt; has been granted.
+To reach &lt;color=#00B9FF&gt;rank 3&lt;/color&gt;, you will need &lt;color=#2DFF00&gt;&lt;b&gt;3&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;Slime Jellies&lt;/b&gt;&lt;/color&gt;.</t>
         </is>
       </c>
     </row>
@@ -4435,7 +4435,7 @@
       <c r="C2" t="inlineStr">
         <is>
           <t>Back again.
-Did you bring &lt;color=#2DFF00&gt;&lt;b&gt;3&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;슬라임 젤리&lt;/b&gt;&lt;/color&gt;?</t>
+Did you bring &lt;color=#2DFF00&gt;&lt;b&gt;3&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;Slime Jellies&lt;/b&gt;&lt;/color&gt;?</t>
         </is>
       </c>
     </row>
@@ -4473,7 +4473,7 @@
       <c r="C4" t="inlineStr">
         <is>
           <t>A new &lt;color=#00B9FF&gt;Rank 3 Permit&lt;/color&gt; has been issued.
-You may now enter &lt;color=#B0FF06&gt;폐허가 된 성소&lt;/color&gt;.
+You may now enter &lt;color=#B0FF06&gt;Ruined Sanctum&lt;/color&gt;.
 Recommended level: &lt;color=#FFFF00&gt;25&lt;/color&gt; or higher.</t>
         </is>
       </c>
@@ -4492,8 +4492,8 @@
       <c r="C5" t="inlineStr">
         <is>
           <t>To reach &lt;color=#00B9FF&gt;rank 4&lt;/color&gt;,
-you will need &lt;color=#2DFF00&gt;&lt;b&gt;5&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;독버섯 갓&lt;/b&gt;&lt;/color&gt;.
-They drop from the creatures of &lt;color=#B0FF06&gt;폐허가 된 성소&lt;/color&gt;.</t>
+you will need &lt;color=#2DFF00&gt;&lt;b&gt;5&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;Toadstool Caps&lt;/b&gt;&lt;/color&gt;.
+They drop from the creatures of &lt;color=#B0FF06&gt;Ruined Sanctum&lt;/color&gt;.</t>
         </is>
       </c>
     </row>
@@ -4556,7 +4556,7 @@
       <c r="C2" t="inlineStr">
         <is>
           <t>Back again.
-Did you bring &lt;color=#2DFF00&gt;&lt;b&gt;5&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;독버섯 갓&lt;/b&gt;&lt;/color&gt;?</t>
+Did you bring &lt;color=#2DFF00&gt;&lt;b&gt;5&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;Toadstool Caps&lt;/b&gt;&lt;/color&gt;?</t>
         </is>
       </c>
     </row>
@@ -4594,7 +4594,7 @@
       <c r="C4" t="inlineStr">
         <is>
           <t>A new &lt;color=#00B9FF&gt;Rank 4 Permit&lt;/color&gt; has been issued.
-You may now enter &lt;color=#B0FF06&gt;가라앉은 숲&lt;/color&gt;.
+You may now enter &lt;color=#B0FF06&gt;Sunken Grove&lt;/color&gt;.
 Recommended level: &lt;color=#FFFF00&gt;37&lt;/color&gt; or higher.</t>
         </is>
       </c>
@@ -4613,8 +4613,8 @@
       <c r="C5" t="inlineStr">
         <is>
           <t>To reach &lt;color=#00B9FF&gt;rank 5&lt;/color&gt;,
-you will need &lt;color=#2DFF00&gt;&lt;b&gt;5&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;까마귀 깃털&lt;/b&gt;&lt;/color&gt;.
-They drop from the creatures of &lt;color=#B0FF06&gt;가라앉은 숲&lt;/color&gt;.</t>
+you will need &lt;color=#2DFF00&gt;&lt;b&gt;5&lt;/b&gt;&lt;/color&gt; &lt;color=#2DFF00&gt;&lt;b&gt;Crow Feathers&lt;/b&gt;&lt;/color&gt;.
+They drop from the creatures of &lt;color=#B0FF06&gt;Sunken Grove&lt;/color&gt;.</t>
         </is>
       </c>
     </row>

</xml_diff>